<commit_message>
Final structue adjustments before submission
</commit_message>
<xml_diff>
--- a/gantt/live/gantt_live.xlsx
+++ b/gantt/live/gantt_live.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="160">
   <si>
     <t>PROJECT TITLE</t>
   </si>
@@ -536,6 +536,12 @@
   </si>
   <si>
     <t>Holiday date</t>
+  </si>
+  <si>
+    <t>In progress</t>
+  </si>
+  <si>
+    <t>Pending</t>
   </si>
 </sst>
 </file>
@@ -578,7 +584,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -655,6 +661,18 @@
       <patternFill patternType="solid">
         <fgColor theme="0"/>
         <bgColor rgb="FFE87BA4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFE699"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8CBAD"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -773,7 +791,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -837,6 +855,9 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1139,7 +1160,7 @@
         <v>6</v>
       </c>
       <c r="K3" s="35">
-        <v>46303</v>
+        <v>46321</v>
       </c>
       <c r="L3" s="35"/>
     </row>
@@ -1303,8 +1324,12 @@
       <c r="E7" s="9">
         <v>46304</v>
       </c>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
+      <c r="F7" s="9">
+        <v>46282</v>
+      </c>
+      <c r="G7" s="9">
+        <v>46304</v>
+      </c>
       <c r="H7" s="7">
         <f>NETWORKDAYS(D7,E7,Holidays!$A$2:$A$1000)</f>
         <v>16</v>
@@ -1599,7 +1624,7 @@
         <v>53</v>
       </c>
       <c r="J12" s="12"/>
-      <c r="K12" s="17"/>
+      <c r="K12" s="12"/>
       <c r="L12" s="17"/>
       <c r="M12" s="15"/>
       <c r="N12" s="12"/>
@@ -1719,7 +1744,7 @@
       <c r="L14" s="12"/>
       <c r="M14" s="15"/>
       <c r="N14" s="12"/>
-      <c r="O14" s="17"/>
+      <c r="O14" s="12"/>
       <c r="P14" s="18"/>
       <c r="Q14" s="15"/>
       <c r="R14" s="12"/>
@@ -1757,8 +1782,12 @@
       <c r="E15" s="9">
         <v>46317</v>
       </c>
-      <c r="F15" s="8"/>
-      <c r="G15" s="8"/>
+      <c r="F15" s="9">
+        <v>46297</v>
+      </c>
+      <c r="G15" s="9">
+        <v>46321</v>
+      </c>
       <c r="H15" s="7">
         <f>NETWORKDAYS(D15,E15,Holidays!$A$2:$A$1000)</f>
         <v>15</v>
@@ -1820,10 +1849,10 @@
       <c r="I16" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="J16" s="19"/>
+      <c r="J16" s="12"/>
       <c r="K16" s="19"/>
       <c r="L16" s="19"/>
-      <c r="M16" s="15"/>
+      <c r="M16" s="20"/>
       <c r="N16" s="12"/>
       <c r="O16" s="12"/>
       <c r="P16" s="15"/>
@@ -1878,8 +1907,8 @@
       <c r="I17" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="J17" s="19"/>
-      <c r="K17" s="19"/>
+      <c r="J17" s="12"/>
+      <c r="K17" s="12"/>
       <c r="L17" s="19"/>
       <c r="M17" s="20"/>
       <c r="N17" s="12"/>
@@ -1923,8 +1952,12 @@
       <c r="E18" s="13">
         <v>46308</v>
       </c>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
+      <c r="F18" s="13">
+        <v>46301</v>
+      </c>
+      <c r="G18" s="13">
+        <v>46303</v>
+      </c>
       <c r="H18" s="12">
         <f>NETWORKDAYS(D18,E18,Holidays!$A$2:$A$1000)</f>
         <v>5</v>
@@ -1935,11 +1968,11 @@
       <c r="J18" s="12"/>
       <c r="K18" s="12"/>
       <c r="L18" s="12"/>
-      <c r="M18" s="40"/>
-      <c r="N18" s="39"/>
-      <c r="O18" s="39"/>
-      <c r="P18" s="40"/>
-      <c r="Q18" s="20"/>
+      <c r="M18" s="20"/>
+      <c r="N18" s="19"/>
+      <c r="O18" s="19"/>
+      <c r="P18" s="15"/>
+      <c r="Q18" s="15"/>
       <c r="R18" s="12"/>
       <c r="S18" s="12"/>
       <c r="T18" s="12"/>
@@ -1978,10 +2011,10 @@
         <v>46308</v>
       </c>
       <c r="F19" s="13">
-        <v>46308</v>
+        <v>46302</v>
       </c>
       <c r="G19" s="13">
-        <v>46308</v>
+        <v>46303</v>
       </c>
       <c r="H19" s="12">
         <f>NETWORKDAYS(D19,E19,Holidays!$A$2:$A$1000)</f>
@@ -1993,13 +2026,13 @@
       <c r="J19" s="12"/>
       <c r="K19" s="12"/>
       <c r="L19" s="12"/>
-      <c r="M19" s="40"/>
-      <c r="N19" s="39"/>
-      <c r="O19" s="39"/>
-      <c r="P19" s="40"/>
-      <c r="Q19" s="20"/>
+      <c r="M19" s="15"/>
+      <c r="N19" s="19"/>
+      <c r="O19" s="19"/>
+      <c r="P19" s="15"/>
+      <c r="Q19" s="15"/>
       <c r="R19" s="12"/>
-      <c r="S19" s="43"/>
+      <c r="S19" s="12"/>
       <c r="T19" s="12"/>
       <c r="U19" s="15"/>
       <c r="V19" s="12"/>
@@ -2036,10 +2069,10 @@
         <v>46308</v>
       </c>
       <c r="F20" s="13">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="G20" s="13">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="H20" s="12">
         <f>NETWORKDAYS(D20,E20,Holidays!$A$2:$A$1000)</f>
@@ -2051,14 +2084,14 @@
       <c r="J20" s="12"/>
       <c r="K20" s="12"/>
       <c r="L20" s="12"/>
-      <c r="M20" s="40"/>
-      <c r="N20" s="39"/>
-      <c r="O20" s="39"/>
-      <c r="P20" s="40"/>
-      <c r="Q20" s="20"/>
-      <c r="R20" s="41"/>
-      <c r="S20" s="44"/>
-      <c r="T20" s="42"/>
+      <c r="M20" s="15"/>
+      <c r="N20" s="12"/>
+      <c r="O20" s="12"/>
+      <c r="P20" s="15"/>
+      <c r="Q20" s="15"/>
+      <c r="R20" s="12"/>
+      <c r="S20" s="12"/>
+      <c r="T20" s="12"/>
       <c r="U20" s="20"/>
       <c r="V20" s="12"/>
       <c r="W20" s="12"/>
@@ -2094,7 +2127,7 @@
         <v>46308</v>
       </c>
       <c r="F21" s="13">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="G21" s="13">
         <v>46315</v>
@@ -2109,16 +2142,16 @@
       <c r="J21" s="12"/>
       <c r="K21" s="12"/>
       <c r="L21" s="12"/>
-      <c r="M21" s="40"/>
-      <c r="N21" s="39"/>
-      <c r="O21" s="39"/>
-      <c r="P21" s="40"/>
-      <c r="Q21" s="20"/>
-      <c r="R21" s="41"/>
-      <c r="S21" s="44"/>
-      <c r="T21" s="42"/>
+      <c r="M21" s="15"/>
+      <c r="N21" s="12"/>
+      <c r="O21" s="12"/>
+      <c r="P21" s="15"/>
+      <c r="Q21" s="15"/>
+      <c r="R21" s="12"/>
+      <c r="S21" s="12"/>
+      <c r="T21" s="12"/>
       <c r="U21" s="20"/>
-      <c r="V21" s="12"/>
+      <c r="V21" s="19"/>
       <c r="W21" s="12"/>
       <c r="X21" s="15"/>
       <c r="Y21" s="12"/>
@@ -2155,7 +2188,7 @@
         <v>46310</v>
       </c>
       <c r="G22" s="13">
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="H22" s="12">
         <f>NETWORKDAYS(D22,E22,Holidays!$A$2:$A$1000)</f>
@@ -2164,23 +2197,23 @@
       <c r="I22" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="J22" s="39"/>
-      <c r="K22" s="39"/>
-      <c r="L22" s="39"/>
-      <c r="M22" s="40"/>
-      <c r="N22" s="39"/>
-      <c r="O22" s="39"/>
-      <c r="P22" s="40"/>
-      <c r="Q22" s="40"/>
-      <c r="R22" s="19"/>
+      <c r="J22" s="12"/>
+      <c r="K22" s="12"/>
+      <c r="L22" s="12"/>
+      <c r="M22" s="15"/>
+      <c r="N22" s="12"/>
+      <c r="O22" s="12"/>
+      <c r="P22" s="15"/>
+      <c r="Q22" s="15"/>
+      <c r="R22" s="12"/>
       <c r="S22" s="19"/>
       <c r="T22" s="19"/>
       <c r="U22" s="20"/>
       <c r="V22" s="19"/>
       <c r="W22" s="19"/>
-      <c r="X22" s="19"/>
+      <c r="X22" s="20"/>
       <c r="Y22" s="19"/>
-      <c r="Z22" s="15"/>
+      <c r="Z22" s="20"/>
       <c r="AA22" s="12"/>
       <c r="AB22" s="12"/>
       <c r="AC22" s="12"/>
@@ -2207,8 +2240,12 @@
       <c r="E23" s="9">
         <v>46317</v>
       </c>
-      <c r="F23" s="8"/>
-      <c r="G23" s="8"/>
+      <c r="F23" s="9">
+        <v>46304</v>
+      </c>
+      <c r="G23" s="9">
+        <v>46321</v>
+      </c>
       <c r="H23" s="7">
         <f>NETWORKDAYS(D23,E23,Holidays!$A$2:$A$1000)</f>
         <v>8</v>
@@ -2258,7 +2295,7 @@
         <v>46310</v>
       </c>
       <c r="F24" s="13">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="G24" s="13">
         <v>46308</v>
@@ -2276,10 +2313,10 @@
       <c r="M24" s="15"/>
       <c r="N24" s="12"/>
       <c r="O24" s="12"/>
-      <c r="P24" s="15"/>
+      <c r="P24" s="21"/>
       <c r="Q24" s="21"/>
-      <c r="R24" s="22"/>
-      <c r="S24" s="22"/>
+      <c r="R24" s="12"/>
+      <c r="S24" s="12"/>
       <c r="T24" s="12"/>
       <c r="U24" s="15"/>
       <c r="V24" s="12"/>
@@ -2374,10 +2411,10 @@
         <v>46314</v>
       </c>
       <c r="F26" s="13">
-        <v>46310</v>
+        <v>46315</v>
       </c>
       <c r="G26" s="13">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="H26" s="12">
         <f>NETWORKDAYS(D26,E26,Holidays!$A$2:$A$1000)</f>
@@ -2393,14 +2430,14 @@
       <c r="N26" s="12"/>
       <c r="O26" s="12"/>
       <c r="P26" s="15"/>
-      <c r="Q26" s="21"/>
-      <c r="R26" s="22"/>
-      <c r="S26" s="22"/>
-      <c r="T26" s="22"/>
-      <c r="U26" s="21"/>
-      <c r="V26" s="12"/>
-      <c r="W26" s="12"/>
-      <c r="X26" s="15"/>
+      <c r="Q26" s="15"/>
+      <c r="R26" s="12"/>
+      <c r="S26" s="12"/>
+      <c r="T26" s="12"/>
+      <c r="U26" s="15"/>
+      <c r="V26" s="22"/>
+      <c r="W26" s="22"/>
+      <c r="X26" s="21"/>
       <c r="Y26" s="12"/>
       <c r="Z26" s="15"/>
       <c r="AA26" s="12"/>
@@ -2435,7 +2472,7 @@
         <v>46317</v>
       </c>
       <c r="G27" s="13">
-        <v>46320</v>
+        <v>46318</v>
       </c>
       <c r="H27" s="12">
         <f>NETWORKDAYS(D27,E27,Holidays!$A$2:$A$1000)</f>
@@ -2456,10 +2493,10 @@
       <c r="S27" s="12"/>
       <c r="T27" s="12"/>
       <c r="U27" s="15"/>
-      <c r="V27" s="22"/>
-      <c r="W27" s="22"/>
+      <c r="V27" s="12"/>
+      <c r="W27" s="12"/>
       <c r="X27" s="21"/>
-      <c r="Y27" s="21"/>
+      <c r="Y27" s="22"/>
       <c r="Z27" s="15"/>
       <c r="AA27" s="12"/>
       <c r="AB27" s="12"/>
@@ -2490,10 +2527,10 @@
         <v>46314</v>
       </c>
       <c r="F28" s="13">
-        <v>46310</v>
+        <v>46315</v>
       </c>
       <c r="G28" s="13">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="H28" s="12">
         <f>NETWORKDAYS(D28,E28,Holidays!$A$2:$A$1000)</f>
@@ -2509,14 +2546,14 @@
       <c r="N28" s="12"/>
       <c r="O28" s="12"/>
       <c r="P28" s="15"/>
-      <c r="Q28" s="21"/>
-      <c r="R28" s="22"/>
-      <c r="S28" s="22"/>
-      <c r="T28" s="22"/>
-      <c r="U28" s="21"/>
-      <c r="V28" s="12"/>
-      <c r="W28" s="12"/>
-      <c r="X28" s="15"/>
+      <c r="Q28" s="15"/>
+      <c r="R28" s="12"/>
+      <c r="S28" s="12"/>
+      <c r="T28" s="12"/>
+      <c r="U28" s="15"/>
+      <c r="V28" s="22"/>
+      <c r="W28" s="22"/>
+      <c r="X28" s="21"/>
       <c r="Y28" s="12"/>
       <c r="Z28" s="15"/>
       <c r="AA28" s="12"/>
@@ -2548,7 +2585,7 @@
         <v>46317</v>
       </c>
       <c r="F29" s="13">
-        <v>46321</v>
+        <v>46317</v>
       </c>
       <c r="G29" s="13">
         <v>46321</v>
@@ -2557,8 +2594,8 @@
         <f>NETWORKDAYS(D29,E29,Holidays!$A$2:$A$1000)</f>
         <v>3</v>
       </c>
-      <c r="I29" s="23" t="s">
-        <v>122</v>
+      <c r="I29" s="14" t="s">
+        <v>53</v>
       </c>
       <c r="J29" s="12"/>
       <c r="K29" s="12"/>
@@ -2572,11 +2609,11 @@
       <c r="S29" s="12"/>
       <c r="T29" s="12"/>
       <c r="U29" s="15"/>
-      <c r="V29" s="22"/>
-      <c r="W29" s="22"/>
+      <c r="V29" s="12"/>
+      <c r="W29" s="12"/>
       <c r="X29" s="21"/>
-      <c r="Y29" s="12"/>
-      <c r="Z29" s="15"/>
+      <c r="Y29" s="22"/>
+      <c r="Z29" s="21"/>
       <c r="AA29" s="12"/>
       <c r="AB29" s="12"/>
       <c r="AC29" s="12"/>
@@ -2603,8 +2640,12 @@
       <c r="E30" s="9">
         <v>46321</v>
       </c>
-      <c r="F30" s="8"/>
-      <c r="G30" s="8"/>
+      <c r="F30" s="9">
+        <v>46310</v>
+      </c>
+      <c r="G30" s="9">
+        <v>46321</v>
+      </c>
       <c r="H30" s="7">
         <f>NETWORKDAYS(D30,E30,Holidays!$A$2:$A$1000)</f>
         <v>7</v>
@@ -2732,6 +2773,7 @@
       <c r="Q32" s="15"/>
       <c r="R32" s="12"/>
       <c r="S32" s="24"/>
+      <c r="T32" s="12"/>
       <c r="U32" s="15"/>
       <c r="V32" s="12"/>
       <c r="W32" s="12"/>
@@ -2770,7 +2812,7 @@
         <v>46317</v>
       </c>
       <c r="G33" s="13">
-        <v>46320</v>
+        <v>46318</v>
       </c>
       <c r="H33" s="12">
         <f>NETWORKDAYS(D33,E33,Holidays!$A$2:$A$1000)</f>
@@ -2790,11 +2832,11 @@
       <c r="R33" s="12"/>
       <c r="S33" s="12"/>
       <c r="T33" s="12"/>
-      <c r="U33" s="37"/>
-      <c r="V33" s="38"/>
-      <c r="W33" s="38"/>
+      <c r="U33" s="15"/>
+      <c r="V33" s="12"/>
+      <c r="W33" s="12"/>
       <c r="X33" s="25"/>
-      <c r="Y33" s="25"/>
+      <c r="Y33" s="24"/>
       <c r="Z33" s="15"/>
       <c r="AA33" s="12"/>
       <c r="AB33" s="12"/>
@@ -2826,7 +2868,7 @@
         <v>46316</v>
       </c>
       <c r="G34" s="13">
-        <v>46320</v>
+        <v>46318</v>
       </c>
       <c r="H34" s="12">
         <f>NETWORKDAYS(D34,E34,Holidays!$A$2:$A$1000)</f>
@@ -2847,10 +2889,10 @@
       <c r="S34" s="12"/>
       <c r="T34" s="12"/>
       <c r="U34" s="15"/>
-      <c r="V34" s="38"/>
+      <c r="V34" s="12"/>
       <c r="W34" s="24"/>
       <c r="X34" s="25"/>
-      <c r="Y34" s="25"/>
+      <c r="Y34" s="24"/>
       <c r="Z34" s="15"/>
       <c r="AA34" s="12"/>
       <c r="AB34" s="12"/>
@@ -2903,10 +2945,10 @@
       <c r="S35" s="12"/>
       <c r="T35" s="12"/>
       <c r="U35" s="15"/>
-      <c r="V35" s="38"/>
+      <c r="V35" s="12"/>
       <c r="W35" s="24"/>
       <c r="X35" s="25"/>
-      <c r="Y35" s="25"/>
+      <c r="Y35" s="24"/>
       <c r="Z35" s="15"/>
       <c r="AA35" s="12"/>
       <c r="AB35" s="12"/>
@@ -2935,7 +2977,7 @@
         <v>46317</v>
       </c>
       <c r="F36" s="13">
-        <v>46321</v>
+        <v>46317</v>
       </c>
       <c r="G36" s="13">
         <v>46321</v>
@@ -2959,10 +3001,10 @@
       <c r="S36" s="12"/>
       <c r="T36" s="12"/>
       <c r="U36" s="15"/>
-      <c r="V36" s="38"/>
-      <c r="W36" s="38"/>
-      <c r="X36" s="37"/>
-      <c r="Y36" s="12"/>
+      <c r="V36" s="12"/>
+      <c r="W36" s="12"/>
+      <c r="X36" s="25"/>
+      <c r="Y36" s="24"/>
       <c r="Z36" s="25"/>
       <c r="AA36" s="12"/>
       <c r="AB36" s="12"/>
@@ -3017,8 +3059,8 @@
       <c r="U37" s="15"/>
       <c r="V37" s="12"/>
       <c r="W37" s="12"/>
-      <c r="X37" s="37"/>
-      <c r="Y37" s="38"/>
+      <c r="X37" s="15"/>
+      <c r="Y37" s="12"/>
       <c r="Z37" s="25"/>
       <c r="AA37" s="12"/>
       <c r="AB37" s="12"/>
@@ -3074,6 +3116,7 @@
       <c r="V38" s="12"/>
       <c r="W38" s="12"/>
       <c r="X38" s="15"/>
+      <c r="Y38" s="12"/>
       <c r="Z38" s="25"/>
       <c r="AA38" s="12"/>
       <c r="AB38" s="12"/>
@@ -3205,8 +3248,8 @@
       <c r="E41" s="13">
         <v>46324</v>
       </c>
-      <c r="F41" s="12"/>
-      <c r="G41" s="12"/>
+      <c r="F41" s="13"/>
+      <c r="G41" s="13"/>
       <c r="H41" s="12">
         <f>NETWORKDAYS(D41,E41,Holidays!$A$2:$A$1000)</f>
         <v>3</v>
@@ -3257,8 +3300,8 @@
       <c r="E42" s="13">
         <v>46325</v>
       </c>
-      <c r="F42" s="12"/>
-      <c r="G42" s="12"/>
+      <c r="F42" s="13"/>
+      <c r="G42" s="13"/>
       <c r="H42" s="12">
         <f>NETWORKDAYS(D42,E42,Holidays!$A$2:$A$1000)</f>
         <v>1</v>
@@ -3309,8 +3352,8 @@
       <c r="E43" s="13">
         <v>46330</v>
       </c>
-      <c r="F43" s="12"/>
-      <c r="G43" s="12"/>
+      <c r="F43" s="13"/>
+      <c r="G43" s="13"/>
       <c r="H43" s="12">
         <f>NETWORKDAYS(D43,E43,Holidays!$A$2:$A$1000)</f>
         <v>2</v>
@@ -3361,8 +3404,8 @@
       <c r="E44" s="13">
         <v>46331</v>
       </c>
-      <c r="F44" s="12"/>
-      <c r="G44" s="12"/>
+      <c r="F44" s="13"/>
+      <c r="G44" s="13"/>
       <c r="H44" s="12">
         <f>NETWORKDAYS(D44,E44,Holidays!$A$2:$A$1000)</f>
         <v>1</v>
@@ -3419,7 +3462,9 @@
       <c r="E46" s="30">
         <v>46331</v>
       </c>
-      <c r="F46" s="29"/>
+      <c r="F46" s="30">
+        <v>46282</v>
+      </c>
       <c r="G46" s="29"/>
       <c r="H46" s="28">
         <f>NETWORKDAYS(D46,E46,Holidays!$A$2:$A$1000)</f>

</xml_diff>